<commit_message>
ordena pestañas por grado 3-5-7-9-11 en Excel y visor
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="10" yWindow="0" windowWidth="19190" windowHeight="10080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worksheet" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worksheet'!$A$1:$E$129</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -452,10 +452,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col width="12.81640625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="16.81640625" customWidth="1" style="1" min="1" max="1"/>
     <col width="16.54296875" customWidth="1" style="1" min="2" max="2"/>
     <col width="9.1796875" customWidth="1" min="3" max="4"/>
     <col width="61.90625" customWidth="1" min="5" max="5"/>
@@ -463,12 +463,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>sede_codigo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>sede_tratada</t>
         </is>
@@ -490,18 +490,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>111001800694</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" t="n">
         <v>111001800694</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -513,18 +513,18 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>111001801047</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" t="n">
         <v>111001800694</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -536,18 +536,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>111001013102</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" t="n">
         <v>111001800694</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -559,18 +559,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>111001083011</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" t="n">
         <v>111001800694</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -582,18 +582,18 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>111001800678</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" t="n">
         <v>111001800678</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -605,18 +605,18 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>111001800643</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" t="n">
         <v>111001800678</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -628,18 +628,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>111001800091</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" t="n">
         <v>111001800678</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -651,18 +651,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>111279000362</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" t="n">
         <v>111001800678</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -674,18 +674,18 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>111001100030</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" t="n">
         <v>111001100030</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -697,18 +697,18 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>111001104281</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" t="n">
         <v>111001100030</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -720,18 +720,18 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>111001012343</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" t="n">
         <v>111001100030</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -743,18 +743,18 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>111001094897</v>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" t="n">
         <v>111001098825</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -766,18 +766,18 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>111001098825</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" t="n">
         <v>111001098825</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -789,18 +789,18 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>111001018252</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" t="n">
         <v>111001098825</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -812,18 +812,18 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>111001018333</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" t="n">
         <v>111001098825</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -835,18 +835,18 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>111001036625</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" t="n">
         <v>111001098922</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -858,18 +858,18 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>111001098965</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" t="n">
         <v>111001098965</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -881,18 +881,18 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>111001045705</v>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" t="n">
         <v>111001098965</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -904,18 +904,18 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>111001045535</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" t="n">
         <v>111001098965</v>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -927,18 +927,18 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>111001030856</v>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" t="n">
         <v>111001098817</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -950,18 +950,18 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>111001098922</v>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" t="n">
         <v>111001098922</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -973,18 +973,18 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>111001104337</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" t="n">
         <v>111001098922</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -996,18 +996,18 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>111001094901</v>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" t="n">
         <v>111001098922</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1019,18 +1019,18 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>111001026069</v>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" t="n">
         <v>111001098931</v>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1042,18 +1042,18 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>111001098817</v>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" t="n">
         <v>111001098817</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1065,18 +1065,18 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>111001046931</v>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" t="n">
         <v>111001098817</v>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1088,18 +1088,18 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>111001012815</v>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" t="n">
         <v>111001098817</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1111,18 +1111,18 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>111001025313</v>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" t="n">
         <v>111001800422</v>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1134,18 +1134,18 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>111001098931</v>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" t="n">
         <v>111001098931</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1157,18 +1157,18 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>111102000265</v>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="B31" t="n">
         <v>111001098931</v>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1180,18 +1180,18 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>111001012441</v>
       </c>
-      <c r="B32" s="1" t="n">
+      <c r="B32" t="n">
         <v>111001098931</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1203,18 +1203,18 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>111001019411</v>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" t="n">
         <v>111001102008</v>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1226,18 +1226,18 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>111001098841</v>
       </c>
-      <c r="B34" s="1" t="n">
+      <c r="B34" t="n">
         <v>111001098841</v>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1249,18 +1249,18 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>111001107760</v>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" t="n">
         <v>111001098841</v>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1272,18 +1272,18 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>111001024686</v>
       </c>
-      <c r="B36" s="1" t="n">
+      <c r="B36" t="n">
         <v>111001098841</v>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1295,18 +1295,18 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>111001017795</v>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" t="n">
         <v>111001098892</v>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1318,18 +1318,18 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>111001100013</v>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" t="n">
         <v>111001100013</v>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1341,18 +1341,18 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>111001107883</v>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" t="n">
         <v>111001100013</v>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1364,18 +1364,18 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>111001801322</v>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" t="n">
         <v>111001100013</v>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1387,18 +1387,18 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>111001015601</v>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" t="n">
         <v>111001104051</v>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1410,18 +1410,18 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>111001800422</v>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" t="n">
         <v>111001800422</v>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1433,18 +1433,18 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>111001104256</v>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" t="n">
         <v>111001800422</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1456,18 +1456,18 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>111001086720</v>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" t="n">
         <v>111001800422</v>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1479,18 +1479,18 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>111001014958</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" t="n">
         <v>111001800554</v>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1502,18 +1502,18 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>111001102008</v>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" t="n">
         <v>111001102008</v>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1525,18 +1525,18 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>111001012033</v>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" t="n">
         <v>111001102008</v>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1548,18 +1548,18 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>111001018309</v>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" t="n">
         <v>111001102008</v>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1571,18 +1571,18 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>111001014745</v>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" t="n">
         <v>111001100056</v>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1594,18 +1594,18 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>111001098850</v>
       </c>
-      <c r="B50" s="1" t="n">
+      <c r="B50" t="n">
         <v>111001098850</v>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1617,18 +1617,18 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>111001801268</v>
       </c>
-      <c r="B51" s="1" t="n">
+      <c r="B51" t="n">
         <v>111001098850</v>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1640,18 +1640,18 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>111001014028</v>
       </c>
-      <c r="B52" s="1" t="n">
+      <c r="B52" t="n">
         <v>111001098850</v>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1663,18 +1663,18 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>111001014591</v>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="B53" t="n">
         <v>111001104043</v>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1686,18 +1686,18 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>111001100021</v>
       </c>
-      <c r="B54" s="1" t="n">
+      <c r="B54" t="n">
         <v>111001100021</v>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1709,18 +1709,18 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>111001801080</v>
       </c>
-      <c r="B55" s="1" t="n">
+      <c r="B55" t="n">
         <v>111001100021</v>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1732,18 +1732,18 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>111850001576</v>
       </c>
-      <c r="B56" s="1" t="n">
+      <c r="B56" t="n">
         <v>111001100021</v>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1755,18 +1755,18 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>111001014214</v>
       </c>
-      <c r="B57" s="1" t="n">
+      <c r="B57" t="n">
         <v>111001098884</v>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1778,18 +1778,18 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>111001098892</v>
       </c>
-      <c r="B58" s="1" t="n">
+      <c r="B58" t="n">
         <v>111001098892</v>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1801,18 +1801,18 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>111001098868</v>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B59" t="n">
         <v>111001098892</v>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1824,18 +1824,18 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>111001012301</v>
       </c>
-      <c r="B60" s="1" t="n">
+      <c r="B60" t="n">
         <v>111001098892</v>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1847,18 +1847,18 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>111001014206</v>
       </c>
-      <c r="B61" s="1" t="n">
+      <c r="B61" t="n">
         <v>111001100064</v>
       </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1870,18 +1870,18 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>111001104051</v>
       </c>
-      <c r="B62" s="1" t="n">
+      <c r="B62" t="n">
         <v>111001104051</v>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1893,18 +1893,18 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>111001801241</v>
       </c>
-      <c r="B63" s="1" t="n">
+      <c r="B63" t="n">
         <v>111001104051</v>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1916,18 +1916,18 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>111001014974</v>
       </c>
-      <c r="B64" s="1" t="n">
+      <c r="B64" t="n">
         <v>111001104051</v>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1939,18 +1939,18 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>111001013374</v>
       </c>
-      <c r="B65" s="1" t="n">
+      <c r="B65" t="n">
         <v>111001098876</v>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -1962,18 +1962,18 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>111001098612</v>
       </c>
-      <c r="B66" s="1" t="n">
+      <c r="B66" t="n">
         <v>111001098612</v>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -1985,18 +1985,18 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>111001015172</v>
       </c>
-      <c r="B67" s="1" t="n">
+      <c r="B67" t="n">
         <v>111001098612</v>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2008,18 +2008,18 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>111001034134</v>
       </c>
-      <c r="B68" s="1" t="n">
+      <c r="B68" t="n">
         <v>111001098612</v>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2031,18 +2031,18 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>111001013153</v>
       </c>
-      <c r="B69" s="1" t="n">
+      <c r="B69" t="n">
         <v>111001800414</v>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2054,18 +2054,18 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>111001800554</v>
       </c>
-      <c r="B70" s="1" t="n">
+      <c r="B70" t="n">
         <v>111001800554</v>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2077,18 +2077,18 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>211001032501</v>
       </c>
-      <c r="B71" s="1" t="n">
+      <c r="B71" t="n">
         <v>111001800554</v>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2100,18 +2100,18 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>111001016039</v>
       </c>
-      <c r="B72" s="1" t="n">
+      <c r="B72" t="n">
         <v>111001800554</v>
       </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2123,18 +2123,18 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>111001012611</v>
       </c>
-      <c r="B73" s="1" t="n">
+      <c r="B73" t="n">
         <v>111001098949</v>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2146,18 +2146,18 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>111001100056</v>
       </c>
-      <c r="B74" s="1" t="n">
+      <c r="B74" t="n">
         <v>111001100056</v>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2169,18 +2169,18 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>111001801276</v>
       </c>
-      <c r="B75" s="1" t="n">
+      <c r="B75" t="n">
         <v>111001100056</v>
       </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2192,18 +2192,18 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>211850000787</v>
       </c>
-      <c r="B76" s="1" t="n">
+      <c r="B76" t="n">
         <v>111001100056</v>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2215,18 +2215,18 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>111001012530</v>
       </c>
-      <c r="B77" s="1" t="n">
+      <c r="B77" t="n">
         <v>111001100072</v>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2238,18 +2238,18 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>111001104043</v>
       </c>
-      <c r="B78" s="1" t="n">
+      <c r="B78" t="n">
         <v>111001104043</v>
       </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2261,18 +2261,18 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>111001104388</v>
       </c>
-      <c r="B79" s="1" t="n">
+      <c r="B79" t="n">
         <v>111001104043</v>
       </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2284,18 +2284,18 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>111265000408</v>
       </c>
-      <c r="B80" s="1" t="n">
+      <c r="B80" t="n">
         <v>111001104043</v>
       </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2307,18 +2307,18 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>111001012360</v>
       </c>
-      <c r="B81" s="1" t="n">
+      <c r="B81" t="n">
         <v>111001800635</v>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2330,18 +2330,18 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>111001098884</v>
       </c>
-      <c r="B82" s="1" t="n">
+      <c r="B82" t="n">
         <v>111001098884</v>
       </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2353,18 +2353,18 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>111001801071</v>
       </c>
-      <c r="B83" s="1" t="n">
+      <c r="B83" t="n">
         <v>111001098884</v>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2376,18 +2376,18 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>111279001296</v>
       </c>
-      <c r="B84" s="1" t="n">
+      <c r="B84" t="n">
         <v>111001098884</v>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2399,18 +2399,18 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>111001011819</v>
       </c>
-      <c r="B85" s="1" t="n">
+      <c r="B85" t="n">
         <v>111001800571</v>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2422,18 +2422,18 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>111001100064</v>
       </c>
-      <c r="B86" s="1" t="n">
+      <c r="B86" t="n">
         <v>111001100064</v>
       </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2445,18 +2445,18 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>111001107794</v>
       </c>
-      <c r="B87" s="1" t="n">
+      <c r="B87" t="n">
         <v>111001100064</v>
       </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2468,18 +2468,18 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>111001041556</v>
       </c>
-      <c r="B88" s="1" t="n">
+      <c r="B88" t="n">
         <v>111001100064</v>
       </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2491,18 +2491,18 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>111001010839</v>
       </c>
-      <c r="B89" s="1" t="n">
+      <c r="B89" t="n">
         <v>111001800431</v>
       </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2514,18 +2514,18 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>111001098876</v>
       </c>
-      <c r="B90" s="1" t="n">
+      <c r="B90" t="n">
         <v>111001098876</v>
       </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2537,18 +2537,18 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>111001016004</v>
       </c>
-      <c r="B91" s="1" t="n">
+      <c r="B91" t="n">
         <v>111001098876</v>
       </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2560,18 +2560,18 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>111001075736</v>
       </c>
-      <c r="B92" s="1" t="n">
+      <c r="B92" t="n">
         <v>111001098876</v>
       </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2583,18 +2583,18 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>111001006122</v>
       </c>
-      <c r="B93" s="1" t="n">
+      <c r="B93" t="n">
         <v>111001800562</v>
       </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2606,18 +2606,18 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>111001800414</v>
       </c>
-      <c r="B94" s="1" t="n">
+      <c r="B94" t="n">
         <v>111001800414</v>
       </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2629,18 +2629,18 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>111001077917</v>
       </c>
-      <c r="B95" s="1" t="n">
+      <c r="B95" t="n">
         <v>111001800414</v>
       </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2652,18 +2652,18 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>111001032433</v>
       </c>
-      <c r="B96" s="1" t="n">
+      <c r="B96" t="n">
         <v>111001800414</v>
       </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2675,18 +2675,18 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>111001098949</v>
       </c>
-      <c r="B97" s="1" t="n">
+      <c r="B97" t="n">
         <v>111001098949</v>
       </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2698,18 +2698,18 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>111001028266</v>
       </c>
-      <c r="B98" s="1" t="n">
+      <c r="B98" t="n">
         <v>111001098949</v>
       </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2721,18 +2721,18 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>111001012483</v>
       </c>
-      <c r="B99" s="1" t="n">
+      <c r="B99" t="n">
         <v>111001098949</v>
       </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2744,18 +2744,18 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>111001100081</v>
       </c>
-      <c r="B100" s="1" t="n">
+      <c r="B100" t="n">
         <v>111001100081</v>
       </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2767,18 +2767,18 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>111001032409</v>
       </c>
-      <c r="B101" s="1" t="n">
+      <c r="B101" t="n">
         <v>111001100081</v>
       </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2790,18 +2790,18 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>111001032450</v>
       </c>
-      <c r="B102" s="1" t="n">
+      <c r="B102" t="n">
         <v>111001100081</v>
       </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2813,18 +2813,18 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" t="n">
         <v>111001100072</v>
       </c>
-      <c r="B103" s="1" t="n">
+      <c r="B103" t="n">
         <v>111001100072</v>
       </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2836,18 +2836,18 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" t="n">
         <v>111001801055</v>
       </c>
-      <c r="B104" s="1" t="n">
+      <c r="B104" t="n">
         <v>111001100072</v>
       </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2859,18 +2859,18 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" t="n">
         <v>111001015911</v>
       </c>
-      <c r="B105" s="1" t="n">
+      <c r="B105" t="n">
         <v>111001100072</v>
       </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2882,18 +2882,18 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" t="n">
         <v>111001800635</v>
       </c>
-      <c r="B106" s="1" t="n">
+      <c r="B106" t="n">
         <v>111001800635</v>
       </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2905,18 +2905,18 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" t="n">
         <v>111001041611</v>
       </c>
-      <c r="B107" s="1" t="n">
+      <c r="B107" t="n">
         <v>111001800635</v>
       </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2928,18 +2928,18 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" t="n">
         <v>111001032395</v>
       </c>
-      <c r="B108" s="1" t="n">
+      <c r="B108" t="n">
         <v>111001800635</v>
       </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2951,18 +2951,18 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" t="n">
         <v>111001800571</v>
       </c>
-      <c r="B109" s="1" t="n">
+      <c r="B109" t="n">
         <v>111001800571</v>
       </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -2974,18 +2974,18 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" t="n">
         <v>111001801101</v>
       </c>
-      <c r="B110" s="1" t="n">
+      <c r="B110" t="n">
         <v>111001800571</v>
       </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -2997,18 +2997,18 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" t="n">
         <v>111001027308</v>
       </c>
-      <c r="B111" s="1" t="n">
+      <c r="B111" t="n">
         <v>111001800571</v>
       </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3020,18 +3020,18 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" t="n">
         <v>111001800431</v>
       </c>
-      <c r="B112" s="1" t="n">
+      <c r="B112" t="n">
         <v>111001800431</v>
       </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3043,18 +3043,18 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" t="n">
         <v>111001034011</v>
       </c>
-      <c r="B113" s="1" t="n">
+      <c r="B113" t="n">
         <v>111001800431</v>
       </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3066,18 +3066,18 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" t="n">
         <v>111001013170</v>
       </c>
-      <c r="B114" s="1" t="n">
+      <c r="B114" t="n">
         <v>111001800431</v>
       </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3089,18 +3089,18 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" t="n">
         <v>111001800562</v>
       </c>
-      <c r="B115" s="1" t="n">
+      <c r="B115" t="n">
         <v>111001800562</v>
       </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3112,18 +3112,18 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" t="n">
         <v>111001801250</v>
       </c>
-      <c r="B116" s="1" t="n">
+      <c r="B116" t="n">
         <v>111001800562</v>
       </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3135,18 +3135,18 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" t="n">
         <v>111001018325</v>
       </c>
-      <c r="B117" s="1" t="n">
+      <c r="B117" t="n">
         <v>111001800562</v>
       </c>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3158,18 +3158,18 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" t="n">
         <v>111001800660</v>
       </c>
-      <c r="B118" s="1" t="n">
+      <c r="B118" t="n">
         <v>111001800660</v>
       </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3181,18 +3181,18 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" t="n">
         <v>111001094439</v>
       </c>
-      <c r="B119" s="1" t="n">
+      <c r="B119" t="n">
         <v>111001800660</v>
       </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3204,18 +3204,18 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" t="n">
         <v>111001034002</v>
       </c>
-      <c r="B120" s="1" t="n">
+      <c r="B120" t="n">
         <v>111001800660</v>
       </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3227,18 +3227,18 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" t="n">
         <v>111001800457</v>
       </c>
-      <c r="B121" s="1" t="n">
+      <c r="B121" t="n">
         <v>111001800457</v>
       </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3250,18 +3250,18 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" t="n">
         <v>111001800163</v>
       </c>
-      <c r="B122" s="1" t="n">
+      <c r="B122" t="n">
         <v>111001800457</v>
       </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3273,18 +3273,18 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" t="n">
         <v>111001106984</v>
       </c>
-      <c r="B123" s="1" t="n">
+      <c r="B123" t="n">
         <v>111001800457</v>
       </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D123" s="2" t="inlineStr">
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3296,18 +3296,18 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" t="n">
         <v>111001800384</v>
       </c>
-      <c r="B124" s="1" t="n">
+      <c r="B124" t="n">
         <v>111001800384</v>
       </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3319,18 +3319,18 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" t="n">
         <v>111001801098</v>
       </c>
-      <c r="B125" s="1" t="n">
+      <c r="B125" t="n">
         <v>111001800384</v>
       </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D125" s="2" t="inlineStr">
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3342,18 +3342,18 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" t="n">
         <v>111001107077</v>
       </c>
-      <c r="B126" s="1" t="n">
+      <c r="B126" t="n">
         <v>111001800384</v>
       </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3365,18 +3365,18 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" t="n">
         <v>111001800392</v>
       </c>
-      <c r="B127" s="1" t="n">
+      <c r="B127" t="n">
         <v>111001800392</v>
       </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D127" s="2" t="inlineStr">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
         <is>
           <t>TRATADO</t>
         </is>
@@ -3388,18 +3388,18 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" t="n">
         <v>111001801314</v>
       </c>
-      <c r="B128" s="1" t="n">
+      <c r="B128" t="n">
         <v>111001800392</v>
       </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3411,18 +3411,18 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" t="n">
         <v>111001107786</v>
       </c>
-      <c r="B129" s="1" t="n">
+      <c r="B129" t="n">
         <v>111001800392</v>
       </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
-      <c r="D129" s="2" t="inlineStr">
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
         <is>
           <t>CONTROL</t>
         </is>
@@ -3430,33 +3430,6 @@
       <c r="E129" t="inlineStr">
         <is>
           <t>COLEGIO NICOLAS BUENAVENTURA (IED)</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>111001800364</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>111001800384</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>COLEGIO JORGE ISAACS (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
actualiza acumulados 28/05/2026 10:49
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223C3082-8E76-4853-930D-02D350FCA289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF4C8C2-96DF-48F1-9C4D-85A4D6A40FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -879,6 +879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -906,7 +907,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>111001800694</v>
       </c>
@@ -923,7 +924,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>111001801047</v>
       </c>
@@ -940,7 +941,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>111001013102</v>
       </c>
@@ -957,7 +958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>111001083011</v>
       </c>
@@ -991,7 +992,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>111001800643</v>
       </c>
@@ -1008,7 +1009,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>111001800091</v>
       </c>
@@ -1025,7 +1026,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>111279000362</v>
       </c>
@@ -1042,7 +1043,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>111001100030</v>
       </c>
@@ -1059,7 +1060,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>111001104281</v>
       </c>
@@ -1076,7 +1077,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>111001012343</v>
       </c>
@@ -1093,7 +1094,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>111001094897</v>
       </c>
@@ -1110,7 +1111,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>111001098825</v>
       </c>
@@ -1127,7 +1128,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>111001018252</v>
       </c>
@@ -1144,7 +1145,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>111001018333</v>
       </c>
@@ -1161,7 +1162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>111001036625</v>
       </c>
@@ -1178,7 +1179,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>111001098965</v>
       </c>
@@ -1195,7 +1196,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>111001045705</v>
       </c>
@@ -1212,7 +1213,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>111001045535</v>
       </c>
@@ -1229,7 +1230,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>111001030856</v>
       </c>
@@ -1246,7 +1247,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>111001098922</v>
       </c>
@@ -1263,7 +1264,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>111001104337</v>
       </c>
@@ -1280,7 +1281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>111001094901</v>
       </c>
@@ -1297,7 +1298,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>111001026069</v>
       </c>
@@ -1314,7 +1315,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>111001098817</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>111001046931</v>
       </c>
@@ -1348,7 +1349,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>111001012815</v>
       </c>
@@ -1365,7 +1366,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>111001025313</v>
       </c>
@@ -1382,7 +1383,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>111001098931</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>111102000265</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>111001012441</v>
       </c>
@@ -1433,7 +1434,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>111001019411</v>
       </c>
@@ -1450,7 +1451,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>111001098841</v>
       </c>
@@ -1467,7 +1468,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>111001107760</v>
       </c>
@@ -1484,7 +1485,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>111001024686</v>
       </c>
@@ -1501,7 +1502,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>111001017795</v>
       </c>
@@ -1518,7 +1519,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>111001100013</v>
       </c>
@@ -1535,7 +1536,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>111001107883</v>
       </c>
@@ -1552,7 +1553,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>111001801322</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>111001015601</v>
       </c>
@@ -1586,7 +1587,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>111001800422</v>
       </c>
@@ -1603,7 +1604,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>111001104256</v>
       </c>
@@ -1620,7 +1621,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>111001086720</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>111001014958</v>
       </c>
@@ -1654,7 +1655,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>111001102008</v>
       </c>
@@ -1671,7 +1672,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>111001012033</v>
       </c>
@@ -1688,7 +1689,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>111001018309</v>
       </c>
@@ -1705,7 +1706,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>111001014745</v>
       </c>
@@ -1722,7 +1723,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>111001098850</v>
       </c>
@@ -1739,7 +1740,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>111001801268</v>
       </c>
@@ -1756,7 +1757,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>111001014028</v>
       </c>
@@ -1773,7 +1774,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>111001014591</v>
       </c>
@@ -1790,7 +1791,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>111001100021</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>111001801080</v>
       </c>
@@ -1824,7 +1825,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>111850001576</v>
       </c>
@@ -1841,7 +1842,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>111001014214</v>
       </c>
@@ -1858,7 +1859,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>111001098892</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>111001098868</v>
       </c>
@@ -1892,7 +1893,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>111001012301</v>
       </c>
@@ -1909,7 +1910,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>111001014206</v>
       </c>
@@ -1926,7 +1927,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>111001104051</v>
       </c>
@@ -1943,7 +1944,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>111001801241</v>
       </c>
@@ -1960,7 +1961,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>111001014974</v>
       </c>
@@ -1977,7 +1978,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>111001013374</v>
       </c>
@@ -1994,7 +1995,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>111001098612</v>
       </c>
@@ -2011,7 +2012,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>111001015172</v>
       </c>
@@ -2028,7 +2029,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>111001034134</v>
       </c>
@@ -2045,7 +2046,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>111001013153</v>
       </c>
@@ -2062,7 +2063,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>111001800554</v>
       </c>
@@ -2079,7 +2080,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>211001032501</v>
       </c>
@@ -2096,7 +2097,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>111001016039</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>111001012611</v>
       </c>
@@ -2130,7 +2131,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>111001100056</v>
       </c>
@@ -2147,7 +2148,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>111001801276</v>
       </c>
@@ -2164,7 +2165,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>211850000787</v>
       </c>
@@ -2181,7 +2182,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>111001012530</v>
       </c>
@@ -2198,7 +2199,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>111001104043</v>
       </c>
@@ -2215,7 +2216,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>111001104388</v>
       </c>
@@ -2232,7 +2233,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>111265000408</v>
       </c>
@@ -2249,7 +2250,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>111001012360</v>
       </c>
@@ -2266,7 +2267,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>111001098884</v>
       </c>
@@ -2283,7 +2284,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>111001801071</v>
       </c>
@@ -2300,7 +2301,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>111279001296</v>
       </c>
@@ -2317,7 +2318,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>111001011819</v>
       </c>
@@ -2334,7 +2335,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>111001100064</v>
       </c>
@@ -2351,7 +2352,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>111001107794</v>
       </c>
@@ -2368,7 +2369,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>111001041556</v>
       </c>
@@ -2385,7 +2386,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>111001010839</v>
       </c>
@@ -2402,7 +2403,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>111001098876</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>111001016004</v>
       </c>
@@ -2436,7 +2437,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>111001075736</v>
       </c>
@@ -2453,7 +2454,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>111001006122</v>
       </c>
@@ -2470,7 +2471,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>111001800414</v>
       </c>
@@ -2487,7 +2488,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>111001077917</v>
       </c>
@@ -2504,7 +2505,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>111001032433</v>
       </c>
@@ -2521,7 +2522,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>111001098949</v>
       </c>
@@ -2538,7 +2539,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>111001028266</v>
       </c>
@@ -2555,7 +2556,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>111001012483</v>
       </c>
@@ -2572,7 +2573,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>111001100081</v>
       </c>
@@ -2589,7 +2590,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>111001032409</v>
       </c>
@@ -2606,7 +2607,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>111001032450</v>
       </c>
@@ -2623,7 +2624,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>111001100072</v>
       </c>
@@ -2640,7 +2641,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>111001801055</v>
       </c>
@@ -2657,7 +2658,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>111001015911</v>
       </c>
@@ -2674,7 +2675,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>111001800635</v>
       </c>
@@ -2691,7 +2692,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>111001041611</v>
       </c>
@@ -2708,7 +2709,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>111001032395</v>
       </c>
@@ -2725,7 +2726,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>111001800571</v>
       </c>
@@ -2742,7 +2743,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>111001801101</v>
       </c>
@@ -2759,7 +2760,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>111001027308</v>
       </c>
@@ -2776,7 +2777,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111001800431</v>
       </c>
@@ -2793,7 +2794,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>111001034011</v>
       </c>
@@ -2810,7 +2811,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>111001013170</v>
       </c>
@@ -2827,7 +2828,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>111001800562</v>
       </c>
@@ -2844,7 +2845,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>111001801250</v>
       </c>
@@ -2861,7 +2862,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>111001018325</v>
       </c>
@@ -2878,7 +2879,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>111001800660</v>
       </c>
@@ -2895,7 +2896,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>111001094439</v>
       </c>
@@ -2912,7 +2913,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>111001034002</v>
       </c>
@@ -2929,7 +2930,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>111001800457</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>111001800163</v>
       </c>
@@ -2963,7 +2964,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>111001106984</v>
       </c>
@@ -2980,7 +2981,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>111001800384</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>111001801098</v>
       </c>
@@ -3014,7 +3015,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>111001107077</v>
       </c>
@@ -3031,7 +3032,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>111001800392</v>
       </c>
@@ -3048,7 +3049,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>111001801314</v>
       </c>
@@ -3065,7 +3066,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>111001107786</v>
       </c>
@@ -3083,7 +3084,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="COLEGIO PARQUES DE BOGOTA (IED)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Remueve P01-P20 del archivo INFORME CLIENTE/ACUMULADO GENERAL.xlsx
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF4C8C2-96DF-48F1-9C4D-85A4D6A40FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C9AC84E-7C3C-42BB-A7F8-1760A0B2DA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$129</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -447,11 +448,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -474,9 +481,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -907,7 +915,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>111001800694</v>
       </c>
@@ -920,7 +928,7 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -975,7 +983,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>111001800678</v>
       </c>
@@ -2552,7 +2560,7 @@
       <c r="D98" t="s">
         <v>7</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E98" s="2" t="s">
         <v>103</v>
       </c>
     </row>
@@ -2756,7 +2764,7 @@
       <c r="D110" t="s">
         <v>7</v>
       </c>
-      <c r="E110" t="s">
+      <c r="E110" s="2" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3087,7 +3095,7 @@
   <autoFilter ref="A1:E129" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="4">
       <filters>
-        <filter val="COLEGIO PARQUES DE BOGOTA (IED)"/>
+        <filter val="COLEGIO LAUREL DE CERA (IED)"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
actualiza acumulados 20/06/2026 17:23
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4B7273-B127-49C7-B5EA-868352F46CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44CF123-2673-4AFB-81F1-ADEBF55BD13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,7 +488,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -886,7 +897,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -898,10 +908,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -914,11 +924,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
         <v>111001800694</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>111001800694</v>
       </c>
       <c r="C2" t="s">
@@ -931,11 +941,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
         <v>111001801047</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>111001800694</v>
       </c>
       <c r="C3" t="s">
@@ -948,11 +958,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
         <v>111001013102</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>111001800694</v>
       </c>
       <c r="C4" t="s">
@@ -965,11 +975,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
         <v>111001083011</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>111001800694</v>
       </c>
       <c r="C5" t="s">
@@ -982,11 +992,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
         <v>111001800678</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>111001800678</v>
       </c>
       <c r="C6" t="s">
@@ -999,11 +1009,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
         <v>111001800643</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>111001800678</v>
       </c>
       <c r="C7" t="s">
@@ -1016,11 +1026,11 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
         <v>111001800091</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>111001800678</v>
       </c>
       <c r="C8" t="s">
@@ -1033,11 +1043,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
         <v>111279000362</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>111001800678</v>
       </c>
       <c r="C9" t="s">
@@ -1050,11 +1060,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A10">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
         <v>111001100030</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>111001100030</v>
       </c>
       <c r="C10" t="s">
@@ -1067,11 +1077,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
         <v>111001104281</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>111001100030</v>
       </c>
       <c r="C11" t="s">
@@ -1084,11 +1094,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A12">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="1">
         <v>111001012343</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>111001100030</v>
       </c>
       <c r="C12" t="s">
@@ -1101,11 +1111,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A13">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
         <v>111001094897</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>111001098825</v>
       </c>
       <c r="C13" t="s">
@@ -1118,11 +1128,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A14">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
         <v>111001098825</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>111001098825</v>
       </c>
       <c r="C14" t="s">
@@ -1135,11 +1145,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A15">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
         <v>111001018252</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>111001098825</v>
       </c>
       <c r="C15" t="s">
@@ -1152,11 +1162,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A16">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
         <v>111001018333</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>111001098825</v>
       </c>
       <c r="C16" t="s">
@@ -1169,11 +1179,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
         <v>111001036625</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>111001098922</v>
       </c>
       <c r="C17" t="s">
@@ -1186,11 +1196,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
         <v>111001098965</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>111001098965</v>
       </c>
       <c r="C18" t="s">
@@ -1203,11 +1213,11 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
         <v>111001045705</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>111001098965</v>
       </c>
       <c r="C19" t="s">
@@ -1220,11 +1230,11 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
         <v>111001045535</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>111001098965</v>
       </c>
       <c r="C20" t="s">
@@ -1237,11 +1247,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="1">
         <v>111001030856</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>111001098817</v>
       </c>
       <c r="C21" t="s">
@@ -1254,11 +1264,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="1">
         <v>111001098922</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="1">
         <v>111001098922</v>
       </c>
       <c r="C22" t="s">
@@ -1271,11 +1281,11 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A23">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
         <v>111001104337</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="1">
         <v>111001098922</v>
       </c>
       <c r="C23" t="s">
@@ -1288,11 +1298,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
         <v>111001094901</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>111001098922</v>
       </c>
       <c r="C24" t="s">
@@ -1305,11 +1315,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
         <v>111001026069</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>111001098931</v>
       </c>
       <c r="C25" t="s">
@@ -1322,11 +1332,11 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
         <v>111001098817</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>111001098817</v>
       </c>
       <c r="C26" t="s">
@@ -1339,11 +1349,11 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A27">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
         <v>111001046931</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>111001098817</v>
       </c>
       <c r="C27" t="s">
@@ -1356,11 +1366,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A28">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
         <v>111001012815</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>111001098817</v>
       </c>
       <c r="C28" t="s">
@@ -1373,11 +1383,11 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A29">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
         <v>111001025313</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>111001800422</v>
       </c>
       <c r="C29" t="s">
@@ -1390,11 +1400,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A30">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
         <v>111001098931</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="1">
         <v>111001098931</v>
       </c>
       <c r="C30" t="s">
@@ -1407,11 +1417,11 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A31">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
         <v>111102000265</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="1">
         <v>111001098931</v>
       </c>
       <c r="C31" t="s">
@@ -1424,11 +1434,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A32">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
         <v>111001012441</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="1">
         <v>111001098931</v>
       </c>
       <c r="C32" t="s">
@@ -1441,11 +1451,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A33">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
         <v>111001019411</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="1">
         <v>111001102008</v>
       </c>
       <c r="C33" t="s">
@@ -1458,11 +1468,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A34">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1">
         <v>111001098841</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="1">
         <v>111001098841</v>
       </c>
       <c r="C34" t="s">
@@ -1475,11 +1485,11 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
         <v>111001107760</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="1">
         <v>111001098841</v>
       </c>
       <c r="C35" t="s">
@@ -1492,11 +1502,11 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A36">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="1">
         <v>111001024686</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="1">
         <v>111001098841</v>
       </c>
       <c r="C36" t="s">
@@ -1509,11 +1519,11 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A37">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
         <v>111001017795</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="1">
         <v>111001098892</v>
       </c>
       <c r="C37" t="s">
@@ -1527,10 +1537,10 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38">
+      <c r="A38" s="1">
         <v>111001100013</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="1">
         <v>111001100013</v>
       </c>
       <c r="C38" t="s">
@@ -1543,11 +1553,11 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A39">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="1">
         <v>111001107883</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>111001100013</v>
       </c>
       <c r="C39" t="s">
@@ -1560,11 +1570,11 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A40">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
         <v>111001801322</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="1">
         <v>111001100013</v>
       </c>
       <c r="C40" t="s">
@@ -1577,11 +1587,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A41">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
         <v>111001015601</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="1">
         <v>111001104051</v>
       </c>
       <c r="C41" t="s">
@@ -1594,11 +1604,11 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A42">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="1">
         <v>111001800422</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="1">
         <v>111001800422</v>
       </c>
       <c r="C42" t="s">
@@ -1611,11 +1621,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A43">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="1">
         <v>111001104256</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="1">
         <v>111001800422</v>
       </c>
       <c r="C43" t="s">
@@ -1628,11 +1638,11 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A44">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" s="1">
         <v>111001086720</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="1">
         <v>111001800422</v>
       </c>
       <c r="C44" t="s">
@@ -1645,11 +1655,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
         <v>111001014958</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="1">
         <v>111001800554</v>
       </c>
       <c r="C45" t="s">
@@ -1662,11 +1672,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A46">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
         <v>111001102008</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="1">
         <v>111001102008</v>
       </c>
       <c r="C46" t="s">
@@ -1679,11 +1689,11 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A47">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="1">
         <v>111001012033</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="1">
         <v>111001102008</v>
       </c>
       <c r="C47" t="s">
@@ -1696,11 +1706,11 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A48">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" s="1">
         <v>111001018309</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="1">
         <v>111001102008</v>
       </c>
       <c r="C48" t="s">
@@ -1713,11 +1723,11 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A49">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="1">
         <v>111001014745</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="1">
         <v>111001100056</v>
       </c>
       <c r="C49" t="s">
@@ -1730,11 +1740,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A50">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="1">
         <v>111001098850</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="1">
         <v>111001098850</v>
       </c>
       <c r="C50" t="s">
@@ -1747,11 +1757,11 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A51">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="1">
         <v>111001801268</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="1">
         <v>111001098850</v>
       </c>
       <c r="C51" t="s">
@@ -1764,11 +1774,11 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A52">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="1">
         <v>111001014028</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="1">
         <v>111001098850</v>
       </c>
       <c r="C52" t="s">
@@ -1781,11 +1791,11 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A53">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" s="1">
         <v>111001014591</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="1">
         <v>111001104043</v>
       </c>
       <c r="C53" t="s">
@@ -1798,11 +1808,11 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A54">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" s="1">
         <v>111001100021</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="1">
         <v>111001100021</v>
       </c>
       <c r="C54" t="s">
@@ -1815,11 +1825,11 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A55">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="1">
         <v>111001801080</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="1">
         <v>111001100021</v>
       </c>
       <c r="C55" t="s">
@@ -1832,11 +1842,11 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A56">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="1">
         <v>111850001576</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="1">
         <v>111001100021</v>
       </c>
       <c r="C56" t="s">
@@ -1849,11 +1859,11 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A57">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
         <v>111001014214</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="1">
         <v>111001098884</v>
       </c>
       <c r="C57" t="s">
@@ -1866,11 +1876,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A58">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
         <v>111001098892</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="1">
         <v>111001098892</v>
       </c>
       <c r="C58" t="s">
@@ -1883,11 +1893,11 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A59">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
         <v>111001098868</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="1">
         <v>111001098892</v>
       </c>
       <c r="C59" t="s">
@@ -1900,11 +1910,11 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A60">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
         <v>111001012301</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="1">
         <v>111001098892</v>
       </c>
       <c r="C60" t="s">
@@ -1917,11 +1927,11 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A61">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
         <v>111001014206</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="1">
         <v>111001100064</v>
       </c>
       <c r="C61" t="s">
@@ -1934,11 +1944,11 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A62">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
         <v>111001104051</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="1">
         <v>111001104051</v>
       </c>
       <c r="C62" t="s">
@@ -1951,11 +1961,11 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A63">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
         <v>111001801241</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="1">
         <v>111001104051</v>
       </c>
       <c r="C63" t="s">
@@ -1968,11 +1978,11 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A64">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
         <v>111001014974</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="1">
         <v>111001104051</v>
       </c>
       <c r="C64" t="s">
@@ -1985,11 +1995,11 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A65">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
         <v>111001013374</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="1">
         <v>111001098876</v>
       </c>
       <c r="C65" t="s">
@@ -2002,11 +2012,11 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A66">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
         <v>111001098612</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="1">
         <v>111001098612</v>
       </c>
       <c r="C66" t="s">
@@ -2019,11 +2029,11 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A67">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
         <v>111001015172</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="1">
         <v>111001098612</v>
       </c>
       <c r="C67" t="s">
@@ -2036,11 +2046,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A68">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
         <v>111001034134</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="1">
         <v>111001098612</v>
       </c>
       <c r="C68" t="s">
@@ -2053,11 +2063,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A69">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
         <v>111001013153</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="1">
         <v>111001800414</v>
       </c>
       <c r="C69" t="s">
@@ -2070,11 +2080,11 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A70">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" s="1">
         <v>111001800554</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="1">
         <v>111001800554</v>
       </c>
       <c r="C70" t="s">
@@ -2087,11 +2097,11 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A71">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" s="1">
         <v>211001032501</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="1">
         <v>111001800554</v>
       </c>
       <c r="C71" t="s">
@@ -2104,11 +2114,11 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A72">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
         <v>111001016039</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="1">
         <v>111001800554</v>
       </c>
       <c r="C72" t="s">
@@ -2121,11 +2131,11 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A73">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
         <v>111001012611</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="1">
         <v>111001098949</v>
       </c>
       <c r="C73" t="s">
@@ -2138,11 +2148,11 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A74">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
         <v>111001100056</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="1">
         <v>111001100056</v>
       </c>
       <c r="C74" t="s">
@@ -2155,11 +2165,11 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A75">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" s="1">
         <v>111001801276</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="1">
         <v>111001100056</v>
       </c>
       <c r="C75" t="s">
@@ -2172,11 +2182,11 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A76">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" s="1">
         <v>211850000787</v>
       </c>
-      <c r="B76">
+      <c r="B76" s="1">
         <v>111001100056</v>
       </c>
       <c r="C76" t="s">
@@ -2189,11 +2199,11 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A77">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" s="1">
         <v>111001012530</v>
       </c>
-      <c r="B77">
+      <c r="B77" s="1">
         <v>111001100072</v>
       </c>
       <c r="C77" t="s">
@@ -2206,11 +2216,11 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A78">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" s="1">
         <v>111001104043</v>
       </c>
-      <c r="B78">
+      <c r="B78" s="1">
         <v>111001104043</v>
       </c>
       <c r="C78" t="s">
@@ -2223,11 +2233,11 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A79">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" s="1">
         <v>111001104388</v>
       </c>
-      <c r="B79">
+      <c r="B79" s="1">
         <v>111001104043</v>
       </c>
       <c r="C79" t="s">
@@ -2240,11 +2250,11 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A80">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" s="1">
         <v>111265000408</v>
       </c>
-      <c r="B80">
+      <c r="B80" s="1">
         <v>111001104043</v>
       </c>
       <c r="C80" t="s">
@@ -2257,11 +2267,11 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A81">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" s="1">
         <v>111001012360</v>
       </c>
-      <c r="B81">
+      <c r="B81" s="1">
         <v>111001800635</v>
       </c>
       <c r="C81" t="s">
@@ -2274,11 +2284,11 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A82">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" s="1">
         <v>111001098884</v>
       </c>
-      <c r="B82">
+      <c r="B82" s="1">
         <v>111001098884</v>
       </c>
       <c r="C82" t="s">
@@ -2291,11 +2301,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A83">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" s="1">
         <v>111001801071</v>
       </c>
-      <c r="B83">
+      <c r="B83" s="1">
         <v>111001098884</v>
       </c>
       <c r="C83" t="s">
@@ -2308,11 +2318,11 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A84">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" s="1">
         <v>111279001296</v>
       </c>
-      <c r="B84">
+      <c r="B84" s="1">
         <v>111001098884</v>
       </c>
       <c r="C84" t="s">
@@ -2325,11 +2335,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A85">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A85" s="1">
         <v>111001011819</v>
       </c>
-      <c r="B85">
+      <c r="B85" s="1">
         <v>111001800571</v>
       </c>
       <c r="C85" t="s">
@@ -2342,11 +2352,11 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A86">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A86" s="1">
         <v>111001100064</v>
       </c>
-      <c r="B86">
+      <c r="B86" s="1">
         <v>111001100064</v>
       </c>
       <c r="C86" t="s">
@@ -2359,11 +2369,11 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A87">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A87" s="1">
         <v>111001107794</v>
       </c>
-      <c r="B87">
+      <c r="B87" s="1">
         <v>111001100064</v>
       </c>
       <c r="C87" t="s">
@@ -2376,11 +2386,11 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A88">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" s="1">
         <v>111001041556</v>
       </c>
-      <c r="B88">
+      <c r="B88" s="1">
         <v>111001100064</v>
       </c>
       <c r="C88" t="s">
@@ -2393,11 +2403,11 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A89">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" s="1">
         <v>111001010839</v>
       </c>
-      <c r="B89">
+      <c r="B89" s="1">
         <v>111001800431</v>
       </c>
       <c r="C89" t="s">
@@ -2410,11 +2420,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A90">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" s="1">
         <v>111001098876</v>
       </c>
-      <c r="B90">
+      <c r="B90" s="1">
         <v>111001098876</v>
       </c>
       <c r="C90" t="s">
@@ -2427,11 +2437,11 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A91">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="1">
         <v>111001016004</v>
       </c>
-      <c r="B91">
+      <c r="B91" s="1">
         <v>111001098876</v>
       </c>
       <c r="C91" t="s">
@@ -2444,11 +2454,11 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A92">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" s="1">
         <v>111001075736</v>
       </c>
-      <c r="B92">
+      <c r="B92" s="1">
         <v>111001098876</v>
       </c>
       <c r="C92" t="s">
@@ -2461,11 +2471,11 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A93">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" s="1">
         <v>111001006122</v>
       </c>
-      <c r="B93">
+      <c r="B93" s="1">
         <v>111001800562</v>
       </c>
       <c r="C93" t="s">
@@ -2478,11 +2488,11 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A94">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="1">
         <v>111001800414</v>
       </c>
-      <c r="B94">
+      <c r="B94" s="1">
         <v>111001800414</v>
       </c>
       <c r="C94" t="s">
@@ -2495,11 +2505,11 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A95">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" s="1">
         <v>111001077917</v>
       </c>
-      <c r="B95">
+      <c r="B95" s="1">
         <v>111001800414</v>
       </c>
       <c r="C95" t="s">
@@ -2512,11 +2522,11 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A96">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="1">
         <v>111001032433</v>
       </c>
-      <c r="B96">
+      <c r="B96" s="1">
         <v>111001800414</v>
       </c>
       <c r="C96" t="s">
@@ -2529,11 +2539,11 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A97">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" s="1">
         <v>111001098949</v>
       </c>
-      <c r="B97">
+      <c r="B97" s="1">
         <v>111001098949</v>
       </c>
       <c r="C97" t="s">
@@ -2546,11 +2556,11 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A98">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A98" s="1">
         <v>111001028266</v>
       </c>
-      <c r="B98">
+      <c r="B98" s="1">
         <v>111001098949</v>
       </c>
       <c r="C98" t="s">
@@ -2563,11 +2573,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A99">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99" s="1">
         <v>111001012483</v>
       </c>
-      <c r="B99">
+      <c r="B99" s="1">
         <v>111001098949</v>
       </c>
       <c r="C99" t="s">
@@ -2580,11 +2590,11 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A100">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" s="1">
         <v>111001100081</v>
       </c>
-      <c r="B100">
+      <c r="B100" s="1">
         <v>111001100081</v>
       </c>
       <c r="C100" t="s">
@@ -2597,11 +2607,11 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A101">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A101" s="1">
         <v>111001032409</v>
       </c>
-      <c r="B101">
+      <c r="B101" s="1">
         <v>111001100081</v>
       </c>
       <c r="C101" t="s">
@@ -2614,11 +2624,11 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A102">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A102" s="1">
         <v>111001032450</v>
       </c>
-      <c r="B102">
+      <c r="B102" s="1">
         <v>111001100081</v>
       </c>
       <c r="C102" t="s">
@@ -2631,11 +2641,11 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A103">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A103" s="1">
         <v>111001100072</v>
       </c>
-      <c r="B103">
+      <c r="B103" s="1">
         <v>111001100072</v>
       </c>
       <c r="C103" t="s">
@@ -2648,11 +2658,11 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A104">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" s="1">
         <v>111001801055</v>
       </c>
-      <c r="B104">
+      <c r="B104" s="1">
         <v>111001100072</v>
       </c>
       <c r="C104" t="s">
@@ -2665,11 +2675,11 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A105">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105" s="1">
         <v>111001015911</v>
       </c>
-      <c r="B105">
+      <c r="B105" s="1">
         <v>111001100072</v>
       </c>
       <c r="C105" t="s">
@@ -2682,11 +2692,11 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A106">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A106" s="1">
         <v>111001800635</v>
       </c>
-      <c r="B106">
+      <c r="B106" s="1">
         <v>111001800635</v>
       </c>
       <c r="C106" t="s">
@@ -2699,11 +2709,11 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A107">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A107" s="1">
         <v>111001041611</v>
       </c>
-      <c r="B107">
+      <c r="B107" s="1">
         <v>111001800635</v>
       </c>
       <c r="C107" t="s">
@@ -2716,11 +2726,11 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A108">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A108" s="1">
         <v>111001032395</v>
       </c>
-      <c r="B108">
+      <c r="B108" s="1">
         <v>111001800635</v>
       </c>
       <c r="C108" t="s">
@@ -2733,11 +2743,11 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A109">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A109" s="1">
         <v>111001800571</v>
       </c>
-      <c r="B109">
+      <c r="B109" s="1">
         <v>111001800571</v>
       </c>
       <c r="C109" t="s">
@@ -2750,11 +2760,11 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A110">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A110" s="1">
         <v>111001801101</v>
       </c>
-      <c r="B110">
+      <c r="B110" s="1">
         <v>111001800571</v>
       </c>
       <c r="C110" t="s">
@@ -2767,11 +2777,11 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A111">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A111" s="1">
         <v>111001027308</v>
       </c>
-      <c r="B111">
+      <c r="B111" s="1">
         <v>111001800571</v>
       </c>
       <c r="C111" t="s">
@@ -2784,11 +2794,11 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A112">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A112" s="1">
         <v>111001800431</v>
       </c>
-      <c r="B112">
+      <c r="B112" s="1">
         <v>111001800431</v>
       </c>
       <c r="C112" t="s">
@@ -2801,11 +2811,11 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A113">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A113" s="1">
         <v>111001034011</v>
       </c>
-      <c r="B113">
+      <c r="B113" s="1">
         <v>111001800431</v>
       </c>
       <c r="C113" t="s">
@@ -2818,11 +2828,11 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A114">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A114" s="1">
         <v>111001013170</v>
       </c>
-      <c r="B114">
+      <c r="B114" s="1">
         <v>111001800431</v>
       </c>
       <c r="C114" t="s">
@@ -2835,11 +2845,11 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A115">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A115" s="1">
         <v>111001800562</v>
       </c>
-      <c r="B115">
+      <c r="B115" s="1">
         <v>111001800562</v>
       </c>
       <c r="C115" t="s">
@@ -2852,11 +2862,11 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A116">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A116" s="1">
         <v>111001801250</v>
       </c>
-      <c r="B116">
+      <c r="B116" s="1">
         <v>111001800562</v>
       </c>
       <c r="C116" t="s">
@@ -2869,11 +2879,11 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A117">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A117" s="1">
         <v>111001018325</v>
       </c>
-      <c r="B117">
+      <c r="B117" s="1">
         <v>111001800562</v>
       </c>
       <c r="C117" t="s">
@@ -2886,11 +2896,11 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A118">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A118" s="1">
         <v>111001800660</v>
       </c>
-      <c r="B118">
+      <c r="B118" s="1">
         <v>111001800660</v>
       </c>
       <c r="C118" t="s">
@@ -2903,11 +2913,11 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A119">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A119" s="1">
         <v>111001094439</v>
       </c>
-      <c r="B119">
+      <c r="B119" s="1">
         <v>111001800660</v>
       </c>
       <c r="C119" t="s">
@@ -2920,11 +2930,11 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A120">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A120" s="1">
         <v>111001034002</v>
       </c>
-      <c r="B120">
+      <c r="B120" s="1">
         <v>111001800660</v>
       </c>
       <c r="C120" t="s">
@@ -2937,11 +2947,11 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A121">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A121" s="1">
         <v>111001800457</v>
       </c>
-      <c r="B121">
+      <c r="B121" s="1">
         <v>111001800457</v>
       </c>
       <c r="C121" t="s">
@@ -2954,11 +2964,11 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A122">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" s="1">
         <v>111001800163</v>
       </c>
-      <c r="B122">
+      <c r="B122" s="1">
         <v>111001800457</v>
       </c>
       <c r="C122" t="s">
@@ -2971,11 +2981,11 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A123">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A123" s="1">
         <v>111001106984</v>
       </c>
-      <c r="B123">
+      <c r="B123" s="1">
         <v>111001800457</v>
       </c>
       <c r="C123" t="s">
@@ -2988,11 +2998,11 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A124">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A124" s="1">
         <v>111001800384</v>
       </c>
-      <c r="B124">
+      <c r="B124" s="1">
         <v>111001800384</v>
       </c>
       <c r="C124" t="s">
@@ -3005,11 +3015,11 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A125">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A125" s="1">
         <v>111001801098</v>
       </c>
-      <c r="B125">
+      <c r="B125" s="1">
         <v>111001800384</v>
       </c>
       <c r="C125" t="s">
@@ -3022,11 +3032,11 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A126">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A126" s="1">
         <v>111001107077</v>
       </c>
-      <c r="B126">
+      <c r="B126" s="1">
         <v>111001800384</v>
       </c>
       <c r="C126" t="s">
@@ -3039,11 +3049,11 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A127">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A127" s="1">
         <v>111001800392</v>
       </c>
-      <c r="B127">
+      <c r="B127" s="1">
         <v>111001800392</v>
       </c>
       <c r="C127" t="s">
@@ -3056,11 +3066,11 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A128">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A128" s="1">
         <v>111001801314</v>
       </c>
-      <c r="B128">
+      <c r="B128" s="1">
         <v>111001800392</v>
       </c>
       <c r="C128" t="s">
@@ -3073,11 +3083,11 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A129">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A129" s="1">
         <v>111001107786</v>
       </c>
-      <c r="B129">
+      <c r="B129" s="1">
         <v>111001800392</v>
       </c>
       <c r="C129" t="s">
@@ -3091,13 +3101,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="COLEGIO BUENAVISTA (IED)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
actualiza acumulados 22/06/2026 08:07
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44CF123-2673-4AFB-81F1-ADEBF55BD13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DAE525-9B8C-4DA7-AE87-A48CF935A332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -480,15 +480,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -897,6 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -908,7 +920,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -924,7 +936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -941,7 +953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -958,7 +970,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -975,7 +987,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -992,7 +1004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1009,7 +1021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1026,7 +1038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1043,7 +1055,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1060,7 +1072,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1077,7 +1089,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1094,7 +1106,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1111,7 +1123,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1128,7 +1140,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1145,7 +1157,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1162,7 +1174,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1179,7 +1191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1196,7 +1208,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1213,7 +1225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1230,7 +1242,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1247,7 +1259,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1264,7 +1276,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1281,7 +1293,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1298,7 +1310,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1315,7 +1327,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1332,7 +1344,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1349,7 +1361,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1366,7 +1378,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1383,7 +1395,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1400,7 +1412,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1417,7 +1429,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1434,7 +1446,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1451,7 +1463,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1468,7 +1480,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1485,7 +1497,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1502,7 +1514,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1519,7 +1531,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1536,7 +1548,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1553,7 +1565,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1570,7 +1582,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1587,7 +1599,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1604,7 +1616,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1621,7 +1633,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1638,7 +1650,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1655,7 +1667,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1672,7 +1684,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1689,7 +1701,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1706,7 +1718,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1723,7 +1735,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1740,7 +1752,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1757,7 +1769,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1774,7 +1786,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1791,7 +1803,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1808,7 +1820,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1825,7 +1837,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1842,7 +1854,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1859,7 +1871,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1876,7 +1888,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1893,7 +1905,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1910,7 +1922,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1927,7 +1939,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1944,7 +1956,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1961,7 +1973,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1978,7 +1990,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -1995,7 +2007,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2012,7 +2024,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2029,7 +2041,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>111001015172</v>
       </c>
@@ -2046,7 +2058,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2063,7 +2075,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2080,7 +2092,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2114,7 +2126,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2131,7 +2143,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2148,7 +2160,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2165,7 +2177,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2182,7 +2194,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2199,7 +2211,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2216,7 +2228,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2233,7 +2245,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2250,7 +2262,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2267,7 +2279,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2284,7 +2296,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2301,7 +2313,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2318,7 +2330,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2335,7 +2347,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2352,7 +2364,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2369,7 +2381,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2386,7 +2398,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2403,7 +2415,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2420,7 +2432,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2437,7 +2449,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2454,7 +2466,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2471,7 +2483,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>111001006122</v>
       </c>
@@ -2488,7 +2500,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2505,7 +2517,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2522,7 +2534,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2539,7 +2551,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2556,7 +2568,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2573,7 +2585,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2590,7 +2602,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2607,7 +2619,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2624,7 +2636,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2641,7 +2653,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2658,7 +2670,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2675,7 +2687,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2692,7 +2704,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2709,7 +2721,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2726,7 +2738,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2743,7 +2755,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2760,7 +2772,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2777,7 +2789,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2794,7 +2806,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2811,7 +2823,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2828,7 +2840,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2845,7 +2857,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2862,7 +2874,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2879,7 +2891,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2896,7 +2908,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2913,7 +2925,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2930,7 +2942,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2947,7 +2959,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2964,7 +2976,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2981,7 +2993,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -2998,7 +3010,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3015,7 +3027,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3032,7 +3044,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3049,7 +3061,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3066,7 +3078,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3083,7 +3095,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3101,8 +3113,17 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="COLEGIO GABRIEL GARCIA MARQUEZ (IED)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
actualiza acumulados 22/06/2026 09:03
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DAE525-9B8C-4DA7-AE87-A48CF935A332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F547951C-1A0E-4BA9-A8D1-EDCEEF0C6A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -908,7 +908,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -936,7 +935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -953,7 +952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -970,7 +969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -987,7 +986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1004,7 +1003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1021,7 +1020,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1055,7 +1054,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1072,7 +1071,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1089,7 +1088,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1123,7 +1122,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1140,7 +1139,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1157,7 +1156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1174,7 +1173,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1191,7 +1190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1208,7 +1207,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1225,7 +1224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1259,7 +1258,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1276,7 +1275,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1310,7 +1309,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1327,7 +1326,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1361,7 +1360,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1395,7 +1394,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1412,7 +1411,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1429,7 +1428,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1446,7 +1445,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1463,7 +1462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1480,7 +1479,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1497,7 +1496,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1531,7 +1530,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1548,7 +1547,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1565,7 +1564,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1582,7 +1581,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1599,7 +1598,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1616,7 +1615,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1633,7 +1632,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1650,7 +1649,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1667,7 +1666,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1684,7 +1683,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1701,7 +1700,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1718,7 +1717,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1735,7 +1734,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1769,7 +1768,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1820,7 +1819,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1837,7 +1836,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1854,7 +1853,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1871,7 +1870,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1888,7 +1887,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1905,7 +1904,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1922,7 +1921,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1939,7 +1938,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1956,7 +1955,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1973,7 +1972,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1990,7 +1989,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2007,7 +2006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2041,7 +2040,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>111001015172</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2075,7 +2074,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2092,7 +2091,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2126,7 +2125,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2143,7 +2142,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2160,7 +2159,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2177,7 +2176,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2194,7 +2193,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2211,7 +2210,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2228,7 +2227,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2245,7 +2244,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2262,7 +2261,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2279,7 +2278,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2296,7 +2295,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2313,7 +2312,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2330,7 +2329,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2347,7 +2346,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2364,7 +2363,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2381,7 +2380,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2398,7 +2397,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2415,7 +2414,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2432,7 +2431,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2449,7 +2448,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2466,7 +2465,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2483,7 +2482,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>111001006122</v>
       </c>
@@ -2500,7 +2499,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2517,7 +2516,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2534,7 +2533,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2551,7 +2550,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2568,7 +2567,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2585,7 +2584,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2602,7 +2601,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2619,7 +2618,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2636,7 +2635,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2653,7 +2652,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2687,7 +2686,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2704,7 +2703,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2721,7 +2720,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2738,7 +2737,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2755,7 +2754,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2772,7 +2771,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2789,7 +2788,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2806,7 +2805,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2823,7 +2822,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2840,7 +2839,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2857,7 +2856,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2891,7 +2890,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2908,7 +2907,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2925,7 +2924,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2942,7 +2941,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2959,7 +2958,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2976,7 +2975,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2993,7 +2992,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3010,7 +3009,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3027,7 +3026,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3044,7 +3043,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3061,7 +3060,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3078,7 +3077,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3095,7 +3094,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3113,18 +3112,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="COLEGIO GABRIEL GARCIA MARQUEZ (IED)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
actualiza acumulados 22/06/2026 12:44
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B89AB5-FD7F-418E-BFC9-B85B09C66EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C197EFC6-7D9F-40E1-AFD1-8056E3B7A439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -908,7 +908,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -936,7 +935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -953,7 +952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -970,7 +969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -987,7 +986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1004,7 +1003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1021,7 +1020,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1055,7 +1054,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1072,7 +1071,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1089,7 +1088,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1123,7 +1122,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1140,7 +1139,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1157,7 +1156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1174,7 +1173,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1191,7 +1190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1208,7 +1207,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1225,7 +1224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1259,7 +1258,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1276,7 +1275,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1310,7 +1309,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1327,7 +1326,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1395,7 +1394,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1412,7 +1411,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1429,7 +1428,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1446,7 +1445,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1463,7 +1462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1480,7 +1479,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1497,7 +1496,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1531,7 +1530,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1548,7 +1547,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1565,7 +1564,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1582,7 +1581,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1599,7 +1598,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1616,7 +1615,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1633,7 +1632,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1650,7 +1649,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1667,7 +1666,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1684,7 +1683,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1701,7 +1700,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1718,7 +1717,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1735,7 +1734,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1769,7 +1768,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1820,7 +1819,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1837,7 +1836,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1854,7 +1853,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1871,7 +1870,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1888,7 +1887,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1905,7 +1904,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1922,7 +1921,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1939,7 +1938,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1956,7 +1955,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1973,7 +1972,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1990,7 +1989,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2007,7 +2006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2041,7 +2040,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>111001015172</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2075,7 +2074,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2092,7 +2091,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2109,7 +2108,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>211001032501</v>
       </c>
@@ -2126,7 +2125,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2143,7 +2142,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2160,7 +2159,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2177,7 +2176,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2194,7 +2193,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2211,7 +2210,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2228,7 +2227,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2245,7 +2244,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2262,7 +2261,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2279,7 +2278,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2296,7 +2295,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2313,7 +2312,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2330,7 +2329,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2347,7 +2346,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2364,7 +2363,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2381,7 +2380,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2398,7 +2397,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2415,7 +2414,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2432,7 +2431,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2449,7 +2448,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2466,7 +2465,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2483,7 +2482,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>111001006122</v>
       </c>
@@ -2500,7 +2499,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2517,7 +2516,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2534,7 +2533,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2551,7 +2550,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2568,7 +2567,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2585,7 +2584,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2602,7 +2601,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2619,7 +2618,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2636,7 +2635,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2653,7 +2652,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2687,7 +2686,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2704,7 +2703,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2721,7 +2720,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2738,7 +2737,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2755,7 +2754,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2772,7 +2771,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2789,7 +2788,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2806,7 +2805,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2823,7 +2822,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2840,7 +2839,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2857,7 +2856,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2891,7 +2890,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2908,7 +2907,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2925,7 +2924,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2942,7 +2941,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2959,7 +2958,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2976,7 +2975,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2993,7 +2992,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3010,7 +3009,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3027,7 +3026,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3044,7 +3043,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3061,7 +3060,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3078,7 +3077,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3095,7 +3094,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3113,13 +3112,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="COLEGIO ATABANZHA (IED)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza acumulados 22/06/2026 15:37
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C197EFC6-7D9F-40E1-AFD1-8056E3B7A439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04330A2-B1AA-4890-8FB2-1F50931F2133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -908,6 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -935,7 +936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -952,7 +953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -969,7 +970,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -986,7 +987,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1003,7 +1004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1020,7 +1021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1037,7 +1038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1054,7 +1055,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1071,7 +1072,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1088,7 +1089,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1105,7 +1106,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1135,11 +1136,11 @@
       <c r="D13" t="s">
         <v>7</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1156,7 +1157,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1173,7 +1174,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1190,7 +1191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1207,7 +1208,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1224,7 +1225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1241,7 +1242,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1258,7 +1259,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1275,7 +1276,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1292,7 +1293,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1309,7 +1310,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1326,7 +1327,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1343,7 +1344,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1360,7 +1361,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1377,7 +1378,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1394,7 +1395,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1411,7 +1412,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1428,7 +1429,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1445,7 +1446,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1462,7 +1463,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1479,7 +1480,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1496,7 +1497,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1513,7 +1514,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1530,7 +1531,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1547,7 +1548,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1564,7 +1565,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1581,7 +1582,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1598,7 +1599,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1615,7 +1616,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1632,7 +1633,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1649,7 +1650,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1683,7 +1684,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1700,7 +1701,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1717,7 +1718,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1734,7 +1735,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1768,7 +1769,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1785,7 +1786,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1802,7 +1803,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1819,7 +1820,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1853,7 +1854,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1870,7 +1871,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1887,7 +1888,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1904,7 +1905,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1921,7 +1922,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1955,7 +1956,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1972,7 +1973,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1989,7 +1990,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2006,7 +2007,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2023,7 +2024,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2040,7 +2041,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>111001015172</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2074,7 +2075,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2091,7 +2092,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2108,7 +2109,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>211001032501</v>
       </c>
@@ -2125,7 +2126,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2142,7 +2143,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2159,7 +2160,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2176,7 +2177,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2193,7 +2194,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2210,7 +2211,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2227,7 +2228,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2244,7 +2245,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2261,7 +2262,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2278,7 +2279,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2295,7 +2296,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2312,7 +2313,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2329,7 +2330,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2346,7 +2347,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2363,7 +2364,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2380,7 +2381,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2397,7 +2398,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2414,7 +2415,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2431,7 +2432,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2448,7 +2449,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2465,7 +2466,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2499,7 +2500,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2516,7 +2517,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2533,7 +2534,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2550,7 +2551,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2567,7 +2568,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2584,7 +2585,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2601,7 +2602,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2618,7 +2619,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2635,7 +2636,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2652,7 +2653,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2669,7 +2670,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2686,7 +2687,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2703,7 +2704,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2720,7 +2721,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2737,7 +2738,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2754,7 +2755,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2771,7 +2772,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2788,7 +2789,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2805,7 +2806,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2822,7 +2823,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2839,7 +2840,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2856,7 +2857,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2873,7 +2874,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2890,7 +2891,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2907,7 +2908,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2924,7 +2925,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2941,7 +2942,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2958,7 +2959,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2975,7 +2976,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2992,7 +2993,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3009,7 +3010,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3026,7 +3027,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3043,7 +3044,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3060,7 +3061,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3077,7 +3078,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3094,7 +3095,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3112,7 +3113,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="111001006122"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza acumulados 24/06/2026 13:49
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04330A2-B1AA-4890-8FB2-1F50931F2133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E54186F-794A-433F-A3EB-E26D228A755A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -908,7 +908,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -936,7 +935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -953,7 +952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -970,7 +969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -987,7 +986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1004,7 +1003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1021,7 +1020,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1055,7 +1054,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1072,7 +1071,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1089,7 +1088,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1123,7 +1122,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1140,7 +1139,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1157,7 +1156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1174,7 +1173,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1191,7 +1190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1208,7 +1207,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1225,7 +1224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1259,7 +1258,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1276,7 +1275,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1310,7 +1309,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1327,7 +1326,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1361,7 +1360,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1395,7 +1394,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1412,7 +1411,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1429,7 +1428,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1446,7 +1445,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1463,7 +1462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1480,7 +1479,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1497,7 +1496,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1531,7 +1530,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1548,7 +1547,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1565,7 +1564,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1582,7 +1581,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1599,7 +1598,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1616,7 +1615,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1633,7 +1632,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1650,7 +1649,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1667,7 +1666,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1684,7 +1683,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1701,7 +1700,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1718,7 +1717,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1735,7 +1734,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1769,7 +1768,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1820,7 +1819,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1837,7 +1836,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1854,7 +1853,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1871,7 +1870,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1888,7 +1887,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1905,7 +1904,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1922,7 +1921,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1939,7 +1938,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1956,7 +1955,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1973,7 +1972,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1990,7 +1989,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2007,7 +2006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2041,7 +2040,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>111001015172</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2075,7 +2074,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2092,7 +2091,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2109,7 +2108,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>211001032501</v>
       </c>
@@ -2126,7 +2125,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2143,7 +2142,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2160,7 +2159,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2177,7 +2176,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2194,7 +2193,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2211,7 +2210,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2228,7 +2227,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2245,7 +2244,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2262,7 +2261,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2279,7 +2278,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2296,7 +2295,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2313,7 +2312,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2330,7 +2329,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2347,7 +2346,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2364,7 +2363,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2381,7 +2380,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2398,7 +2397,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2415,7 +2414,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2432,7 +2431,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2449,7 +2448,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2466,7 +2465,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2500,7 +2499,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2517,7 +2516,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2534,7 +2533,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2551,7 +2550,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2568,7 +2567,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2585,7 +2584,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2602,7 +2601,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2619,7 +2618,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2636,7 +2635,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2653,7 +2652,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2687,7 +2686,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2704,7 +2703,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2721,7 +2720,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2738,7 +2737,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2755,7 +2754,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2772,7 +2771,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2789,7 +2788,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2806,7 +2805,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2823,7 +2822,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2840,7 +2839,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2857,7 +2856,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2891,7 +2890,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2908,7 +2907,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2925,7 +2924,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2942,7 +2941,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2959,7 +2958,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2976,7 +2975,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2993,7 +2992,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3010,7 +3009,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3027,7 +3026,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3044,7 +3043,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3061,7 +3060,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3078,7 +3077,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3095,7 +3094,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3113,13 +3112,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="111001006122"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza acumulados 24/06/2026 17:54
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E54186F-794A-433F-A3EB-E26D228A755A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2A07D5-93F1-4D87-8E6C-9A2D80413508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$129</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -460,12 +460,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -480,11 +486,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -908,6 +915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -925,17 +933,17 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -952,7 +960,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -969,7 +977,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -986,7 +994,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1003,7 +1011,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1020,7 +1028,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1037,7 +1045,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1054,7 +1062,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1071,7 +1079,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1088,7 +1096,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1105,7 +1113,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1122,7 +1130,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1139,7 +1147,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1156,7 +1164,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1173,7 +1181,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1190,7 +1198,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1207,7 +1215,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1224,7 +1232,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1241,7 +1249,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1258,7 +1266,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1275,7 +1283,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1292,7 +1300,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1309,7 +1317,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1326,7 +1334,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1343,7 +1351,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1360,7 +1368,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1377,7 +1385,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1394,7 +1402,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1411,7 +1419,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1428,7 +1436,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1445,7 +1453,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1462,7 +1470,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1479,7 +1487,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1496,7 +1504,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1513,7 +1521,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1530,7 +1538,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1547,7 +1555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1564,7 +1572,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1581,7 +1589,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1598,7 +1606,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1615,7 +1623,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1632,7 +1640,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1649,7 +1657,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1666,7 +1674,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1683,7 +1691,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1700,7 +1708,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1717,7 +1725,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1734,7 +1742,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1751,7 +1759,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1768,7 +1776,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1785,7 +1793,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1802,7 +1810,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1819,7 +1827,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1836,7 +1844,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1853,7 +1861,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1870,7 +1878,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1887,7 +1895,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1904,7 +1912,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1921,7 +1929,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1938,7 +1946,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1955,7 +1963,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1972,7 +1980,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1989,7 +1997,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2006,7 +2014,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2023,7 +2031,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2057,7 +2065,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2074,7 +2082,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2091,7 +2099,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2108,7 +2116,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>211001032501</v>
       </c>
@@ -2125,7 +2133,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2142,7 +2150,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2159,7 +2167,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2176,7 +2184,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2193,7 +2201,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2210,7 +2218,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2227,7 +2235,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2244,7 +2252,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2261,7 +2269,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2278,7 +2286,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2295,7 +2303,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2312,7 +2320,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2329,7 +2337,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2346,7 +2354,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2363,7 +2371,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2380,7 +2388,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2397,7 +2405,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2414,7 +2422,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2431,7 +2439,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2448,7 +2456,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2465,7 +2473,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2482,7 +2490,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>111001006122</v>
       </c>
@@ -2499,7 +2507,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2516,7 +2524,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2533,7 +2541,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2550,7 +2558,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2567,7 +2575,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2584,7 +2592,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2601,7 +2609,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2618,7 +2626,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2635,7 +2643,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2652,7 +2660,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2669,7 +2677,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2686,7 +2694,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2703,7 +2711,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2720,7 +2728,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2737,7 +2745,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2754,7 +2762,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2771,7 +2779,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2788,7 +2796,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2805,7 +2813,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2822,7 +2830,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2839,7 +2847,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2856,7 +2864,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2873,7 +2881,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2890,7 +2898,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2907,7 +2915,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2924,7 +2932,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2941,7 +2949,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2958,7 +2966,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2975,7 +2983,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -2992,7 +3000,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3009,7 +3017,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3026,7 +3034,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3043,7 +3051,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3060,7 +3068,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3077,7 +3085,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3094,7 +3102,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3112,7 +3120,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="COLEGIO ALEJANDRO OBREGON (IED)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza acumulados 24/06/2026 18:58
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2A07D5-93F1-4D87-8E6C-9A2D80413508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FD6836-4554-4809-BFBC-B2D21FB80B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -915,7 +915,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -943,7 +942,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>111001800694</v>
       </c>
@@ -960,7 +959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>111001801047</v>
       </c>
@@ -977,7 +976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>111001013102</v>
       </c>
@@ -994,7 +993,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>111001083011</v>
       </c>
@@ -1011,7 +1010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>111001800678</v>
       </c>
@@ -1028,7 +1027,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>111001800643</v>
       </c>
@@ -1045,7 +1044,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>111001800091</v>
       </c>
@@ -1062,7 +1061,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>111279000362</v>
       </c>
@@ -1079,7 +1078,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>111001100030</v>
       </c>
@@ -1096,7 +1095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>111001104281</v>
       </c>
@@ -1113,7 +1112,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>111001012343</v>
       </c>
@@ -1130,7 +1129,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>111001094897</v>
       </c>
@@ -1147,7 +1146,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>111001098825</v>
       </c>
@@ -1164,7 +1163,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>111001018252</v>
       </c>
@@ -1181,7 +1180,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>111001018333</v>
       </c>
@@ -1198,7 +1197,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>111001036625</v>
       </c>
@@ -1215,7 +1214,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>111001098965</v>
       </c>
@@ -1232,7 +1231,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>111001045705</v>
       </c>
@@ -1249,7 +1248,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>111001045535</v>
       </c>
@@ -1266,7 +1265,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>111001030856</v>
       </c>
@@ -1283,7 +1282,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>111001098922</v>
       </c>
@@ -1300,7 +1299,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>111001104337</v>
       </c>
@@ -1317,7 +1316,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>111001094901</v>
       </c>
@@ -1334,7 +1333,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>111001026069</v>
       </c>
@@ -1351,7 +1350,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>111001098817</v>
       </c>
@@ -1368,7 +1367,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>111001046931</v>
       </c>
@@ -1385,7 +1384,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>111001012815</v>
       </c>
@@ -1402,7 +1401,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>111001025313</v>
       </c>
@@ -1419,7 +1418,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>111001098931</v>
       </c>
@@ -1436,7 +1435,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>111102000265</v>
       </c>
@@ -1453,7 +1452,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>111001012441</v>
       </c>
@@ -1470,7 +1469,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>111001019411</v>
       </c>
@@ -1487,7 +1486,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>111001098841</v>
       </c>
@@ -1504,7 +1503,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>111001107760</v>
       </c>
@@ -1521,7 +1520,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>111001024686</v>
       </c>
@@ -1538,7 +1537,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>111001017795</v>
       </c>
@@ -1555,7 +1554,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>111001100013</v>
       </c>
@@ -1572,7 +1571,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>111001107883</v>
       </c>
@@ -1589,7 +1588,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>111001801322</v>
       </c>
@@ -1606,7 +1605,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>111001015601</v>
       </c>
@@ -1623,7 +1622,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>111001800422</v>
       </c>
@@ -1640,7 +1639,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>111001104256</v>
       </c>
@@ -1657,7 +1656,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>111001086720</v>
       </c>
@@ -1674,7 +1673,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>111001014958</v>
       </c>
@@ -1691,7 +1690,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>111001102008</v>
       </c>
@@ -1708,7 +1707,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>111001012033</v>
       </c>
@@ -1725,7 +1724,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>111001018309</v>
       </c>
@@ -1742,7 +1741,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>111001014745</v>
       </c>
@@ -1759,7 +1758,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>111001098850</v>
       </c>
@@ -1776,7 +1775,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>111001801268</v>
       </c>
@@ -1793,7 +1792,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>111001014028</v>
       </c>
@@ -1810,7 +1809,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>111001014591</v>
       </c>
@@ -1827,7 +1826,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>111001100021</v>
       </c>
@@ -1844,7 +1843,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>111001801080</v>
       </c>
@@ -1861,7 +1860,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>111850001576</v>
       </c>
@@ -1878,7 +1877,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>111001014214</v>
       </c>
@@ -1895,7 +1894,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>111001098892</v>
       </c>
@@ -1912,7 +1911,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>111001098868</v>
       </c>
@@ -1929,7 +1928,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>111001012301</v>
       </c>
@@ -1946,7 +1945,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>111001014206</v>
       </c>
@@ -1963,7 +1962,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>111001104051</v>
       </c>
@@ -1980,7 +1979,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>111001801241</v>
       </c>
@@ -1997,7 +1996,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>111001014974</v>
       </c>
@@ -2014,7 +2013,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>111001013374</v>
       </c>
@@ -2031,7 +2030,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>111001098612</v>
       </c>
@@ -2065,7 +2064,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>111001034134</v>
       </c>
@@ -2082,7 +2081,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>111001013153</v>
       </c>
@@ -2099,7 +2098,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>111001800554</v>
       </c>
@@ -2116,7 +2115,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>211001032501</v>
       </c>
@@ -2133,7 +2132,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>111001016039</v>
       </c>
@@ -2150,7 +2149,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>111001012611</v>
       </c>
@@ -2167,7 +2166,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>111001100056</v>
       </c>
@@ -2184,7 +2183,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>111001801276</v>
       </c>
@@ -2201,7 +2200,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>211850000787</v>
       </c>
@@ -2218,7 +2217,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>111001012530</v>
       </c>
@@ -2235,7 +2234,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>111001104043</v>
       </c>
@@ -2252,7 +2251,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>111001104388</v>
       </c>
@@ -2269,7 +2268,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>111265000408</v>
       </c>
@@ -2286,7 +2285,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>111001012360</v>
       </c>
@@ -2303,7 +2302,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>111001098884</v>
       </c>
@@ -2320,7 +2319,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>111001801071</v>
       </c>
@@ -2337,7 +2336,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>111279001296</v>
       </c>
@@ -2354,7 +2353,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>111001011819</v>
       </c>
@@ -2371,7 +2370,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>111001100064</v>
       </c>
@@ -2388,7 +2387,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>111001107794</v>
       </c>
@@ -2405,7 +2404,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>111001041556</v>
       </c>
@@ -2422,7 +2421,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>111001010839</v>
       </c>
@@ -2439,7 +2438,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>111001098876</v>
       </c>
@@ -2456,7 +2455,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>111001016004</v>
       </c>
@@ -2473,7 +2472,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>111001075736</v>
       </c>
@@ -2490,7 +2489,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>111001006122</v>
       </c>
@@ -2507,7 +2506,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>111001800414</v>
       </c>
@@ -2524,7 +2523,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>111001077917</v>
       </c>
@@ -2541,7 +2540,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>111001032433</v>
       </c>
@@ -2558,7 +2557,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>111001098949</v>
       </c>
@@ -2575,7 +2574,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>111001028266</v>
       </c>
@@ -2592,7 +2591,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>111001012483</v>
       </c>
@@ -2609,7 +2608,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>111001100081</v>
       </c>
@@ -2626,7 +2625,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>111001032409</v>
       </c>
@@ -2643,7 +2642,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>111001032450</v>
       </c>
@@ -2660,7 +2659,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>111001100072</v>
       </c>
@@ -2677,7 +2676,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>111001801055</v>
       </c>
@@ -2694,7 +2693,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>111001015911</v>
       </c>
@@ -2711,7 +2710,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>111001800635</v>
       </c>
@@ -2728,7 +2727,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>111001041611</v>
       </c>
@@ -2745,7 +2744,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>111001032395</v>
       </c>
@@ -2762,7 +2761,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>111001800571</v>
       </c>
@@ -2779,7 +2778,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>111001801101</v>
       </c>
@@ -2796,7 +2795,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>111001027308</v>
       </c>
@@ -2813,7 +2812,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111001800431</v>
       </c>
@@ -2830,7 +2829,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>111001034011</v>
       </c>
@@ -2847,7 +2846,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>111001013170</v>
       </c>
@@ -2864,7 +2863,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>111001800562</v>
       </c>
@@ -2881,7 +2880,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>111001801250</v>
       </c>
@@ -2898,7 +2897,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>111001018325</v>
       </c>
@@ -2915,7 +2914,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>111001800660</v>
       </c>
@@ -2932,7 +2931,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>111001094439</v>
       </c>
@@ -2949,7 +2948,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>111001034002</v>
       </c>
@@ -2966,7 +2965,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>111001800457</v>
       </c>
@@ -2983,7 +2982,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>111001800163</v>
       </c>
@@ -3000,7 +2999,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>111001106984</v>
       </c>
@@ -3017,7 +3016,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>111001800384</v>
       </c>
@@ -3034,7 +3033,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>111001801098</v>
       </c>
@@ -3051,7 +3050,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>111001107077</v>
       </c>
@@ -3068,7 +3067,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>111001800392</v>
       </c>
@@ -3085,7 +3084,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>111001801314</v>
       </c>
@@ -3102,7 +3101,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>111001107786</v>
       </c>
@@ -3120,13 +3119,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="COLEGIO ALEJANDRO OBREGON (IED)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
actualiza acumulados 25/06/2026 10:08
</commit_message>
<xml_diff>
--- a/Seguimiento.xlsx
+++ b/Seguimiento.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FD6836-4554-4809-BFBC-B2D21FB80B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434E657E-4ACF-4FA2-BB26-E357F543333C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$E$129</definedName>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="135">
   <si>
     <t>sede_codigo</t>
   </si>
@@ -447,7 +449,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -459,8 +461,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -471,6 +485,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -486,17 +506,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3121,12 +3159,1528 @@
   </sheetData>
   <autoFilter ref="A1:E129" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60200415-090D-441E-A131-651DD9159955}">
+  <dimension ref="A1:C129"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="61.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>111001800694</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>111001801047</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>111001013102</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
+        <v>111001083011</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>111001800678</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>111001800643</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>111001800091</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>111279000362</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>111001100030</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
+        <v>111001104281</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="1">
+        <v>111001012343</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
+        <v>111001094897</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
+        <v>111001098825</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
+        <v>111001018252</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>111001018333</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
+        <v>111001036625</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
+        <v>111001098965</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
+        <v>111001045705</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
+        <v>111001045535</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="1">
+        <v>111001030856</v>
+      </c>
+      <c r="B21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="1">
+        <v>111001098922</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
+        <v>111001104337</v>
+      </c>
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
+        <v>111001094901</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
+        <v>111001026069</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
+        <v>111001098817</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
+        <v>111001046931</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
+        <v>111001012815</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
+        <v>111001025313</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
+        <v>111001098931</v>
+      </c>
+      <c r="B30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
+        <v>111102000265</v>
+      </c>
+      <c r="B31" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
+        <v>111001012441</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
+        <v>111001019411</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="1">
+        <v>111001098841</v>
+      </c>
+      <c r="B34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
+        <v>111001107760</v>
+      </c>
+      <c r="B35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="1">
+        <v>111001024686</v>
+      </c>
+      <c r="B36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
+        <v>111001017795</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="1">
+        <v>111001100013</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="1">
+        <v>111001107883</v>
+      </c>
+      <c r="B39" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
+        <v>111001801322</v>
+      </c>
+      <c r="B40" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
+        <v>111001015601</v>
+      </c>
+      <c r="B41" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="1">
+        <v>111001800422</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="1">
+        <v>111001104256</v>
+      </c>
+      <c r="B43" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="1">
+        <v>111001086720</v>
+      </c>
+      <c r="B44" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
+        <v>111001014958</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
+        <v>111001102008</v>
+      </c>
+      <c r="B46" t="s">
+        <v>5</v>
+      </c>
+      <c r="C46" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="1">
+        <v>111001012033</v>
+      </c>
+      <c r="B47" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="1">
+        <v>111001018309</v>
+      </c>
+      <c r="B48" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="1">
+        <v>111001014745</v>
+      </c>
+      <c r="B49" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="1">
+        <v>111001098850</v>
+      </c>
+      <c r="B50" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="1">
+        <v>111001801268</v>
+      </c>
+      <c r="B51" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="1">
+        <v>111001014028</v>
+      </c>
+      <c r="B52" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="1">
+        <v>111001014591</v>
+      </c>
+      <c r="B53" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="1">
+        <v>111001100021</v>
+      </c>
+      <c r="B54" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="1">
+        <v>111001801080</v>
+      </c>
+      <c r="B55" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="1">
+        <v>111850001576</v>
+      </c>
+      <c r="B56" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
+        <v>111001014214</v>
+      </c>
+      <c r="B57" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
+        <v>111001098892</v>
+      </c>
+      <c r="B58" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
+        <v>111001098868</v>
+      </c>
+      <c r="B59" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
+        <v>111001012301</v>
+      </c>
+      <c r="B60" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
+        <v>111001014206</v>
+      </c>
+      <c r="B61" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
+        <v>111001104051</v>
+      </c>
+      <c r="B62" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
+        <v>111001801241</v>
+      </c>
+      <c r="B63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
+        <v>111001014974</v>
+      </c>
+      <c r="B64" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
+        <v>111001013374</v>
+      </c>
+      <c r="B65" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
+        <v>111001098612</v>
+      </c>
+      <c r="B66" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
+        <v>111001015172</v>
+      </c>
+      <c r="B67" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
+        <v>111001034134</v>
+      </c>
+      <c r="B68" t="s">
+        <v>7</v>
+      </c>
+      <c r="C68" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
+        <v>111001013153</v>
+      </c>
+      <c r="B69" t="s">
+        <v>7</v>
+      </c>
+      <c r="C69" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="1">
+        <v>111001800554</v>
+      </c>
+      <c r="B70" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" s="1">
+        <v>211001032501</v>
+      </c>
+      <c r="B71" t="s">
+        <v>7</v>
+      </c>
+      <c r="C71" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
+        <v>111001016039</v>
+      </c>
+      <c r="B72" t="s">
+        <v>7</v>
+      </c>
+      <c r="C72" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
+        <v>111001012611</v>
+      </c>
+      <c r="B73" t="s">
+        <v>7</v>
+      </c>
+      <c r="C73" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
+        <v>111001100056</v>
+      </c>
+      <c r="B74" t="s">
+        <v>5</v>
+      </c>
+      <c r="C74" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" s="1">
+        <v>111001801276</v>
+      </c>
+      <c r="B75" t="s">
+        <v>7</v>
+      </c>
+      <c r="C75" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" s="1">
+        <v>211850000787</v>
+      </c>
+      <c r="B76" t="s">
+        <v>7</v>
+      </c>
+      <c r="C76" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" s="1">
+        <v>111001012530</v>
+      </c>
+      <c r="B77" t="s">
+        <v>7</v>
+      </c>
+      <c r="C77" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" s="1">
+        <v>111001104043</v>
+      </c>
+      <c r="B78" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" s="1">
+        <v>111001104388</v>
+      </c>
+      <c r="B79" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" s="1">
+        <v>111265000408</v>
+      </c>
+      <c r="B80" t="s">
+        <v>7</v>
+      </c>
+      <c r="C80" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" s="1">
+        <v>111001012360</v>
+      </c>
+      <c r="B81" t="s">
+        <v>7</v>
+      </c>
+      <c r="C81" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" s="1">
+        <v>111001098884</v>
+      </c>
+      <c r="B82" t="s">
+        <v>5</v>
+      </c>
+      <c r="C82" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" s="1">
+        <v>111001801071</v>
+      </c>
+      <c r="B83" t="s">
+        <v>7</v>
+      </c>
+      <c r="C83" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" s="1">
+        <v>111279001296</v>
+      </c>
+      <c r="B84" t="s">
+        <v>7</v>
+      </c>
+      <c r="C84" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" s="1">
+        <v>111001011819</v>
+      </c>
+      <c r="B85" t="s">
+        <v>7</v>
+      </c>
+      <c r="C85" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" s="1">
+        <v>111001100064</v>
+      </c>
+      <c r="B86" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" s="1">
+        <v>111001107794</v>
+      </c>
+      <c r="B87" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" s="1">
+        <v>111001041556</v>
+      </c>
+      <c r="B88" t="s">
+        <v>7</v>
+      </c>
+      <c r="C88" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" s="1">
+        <v>111001010839</v>
+      </c>
+      <c r="B89" t="s">
+        <v>7</v>
+      </c>
+      <c r="C89" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90" s="1">
+        <v>111001098876</v>
+      </c>
+      <c r="B90" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91" s="1">
+        <v>111001016004</v>
+      </c>
+      <c r="B91" t="s">
+        <v>7</v>
+      </c>
+      <c r="C91" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92" s="1">
+        <v>111001075736</v>
+      </c>
+      <c r="B92" t="s">
+        <v>7</v>
+      </c>
+      <c r="C92" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93" s="1">
+        <v>111001006122</v>
+      </c>
+      <c r="B93" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" s="1">
+        <v>111001800414</v>
+      </c>
+      <c r="B94" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" s="1">
+        <v>111001077917</v>
+      </c>
+      <c r="B95" t="s">
+        <v>7</v>
+      </c>
+      <c r="C95" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" s="1">
+        <v>111001032433</v>
+      </c>
+      <c r="B96" t="s">
+        <v>7</v>
+      </c>
+      <c r="C96" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" s="1">
+        <v>111001098949</v>
+      </c>
+      <c r="B97" t="s">
+        <v>5</v>
+      </c>
+      <c r="C97" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" s="1">
+        <v>111001028266</v>
+      </c>
+      <c r="B98" t="s">
+        <v>7</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" s="1">
+        <v>111001012483</v>
+      </c>
+      <c r="B99" t="s">
+        <v>7</v>
+      </c>
+      <c r="C99" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" s="1">
+        <v>111001100081</v>
+      </c>
+      <c r="B100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C100" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" s="1">
+        <v>111001032409</v>
+      </c>
+      <c r="B101" t="s">
+        <v>7</v>
+      </c>
+      <c r="C101" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" s="1">
+        <v>111001032450</v>
+      </c>
+      <c r="B102" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" s="1">
+        <v>111001100072</v>
+      </c>
+      <c r="B103" t="s">
+        <v>5</v>
+      </c>
+      <c r="C103" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A104" s="1">
+        <v>111001801055</v>
+      </c>
+      <c r="B104" t="s">
+        <v>7</v>
+      </c>
+      <c r="C104" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A105" s="1">
+        <v>111001015911</v>
+      </c>
+      <c r="B105" t="s">
+        <v>7</v>
+      </c>
+      <c r="C105" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A106" s="1">
+        <v>111001800635</v>
+      </c>
+      <c r="B106" t="s">
+        <v>5</v>
+      </c>
+      <c r="C106" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A107" s="1">
+        <v>111001041611</v>
+      </c>
+      <c r="B107" t="s">
+        <v>7</v>
+      </c>
+      <c r="C107" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A108" s="1">
+        <v>111001032395</v>
+      </c>
+      <c r="B108" t="s">
+        <v>7</v>
+      </c>
+      <c r="C108" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A109" s="1">
+        <v>111001800571</v>
+      </c>
+      <c r="B109" t="s">
+        <v>5</v>
+      </c>
+      <c r="C109" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A110" s="1">
+        <v>111001801101</v>
+      </c>
+      <c r="B110" t="s">
+        <v>7</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A111" s="1">
+        <v>111001027308</v>
+      </c>
+      <c r="B111" t="s">
+        <v>7</v>
+      </c>
+      <c r="C111" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A112" s="1">
+        <v>111001800431</v>
+      </c>
+      <c r="B112" t="s">
+        <v>5</v>
+      </c>
+      <c r="C112" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" s="1">
+        <v>111001034011</v>
+      </c>
+      <c r="B113" t="s">
+        <v>7</v>
+      </c>
+      <c r="C113" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" s="1">
+        <v>111001013170</v>
+      </c>
+      <c r="B114" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" s="1">
+        <v>111001800562</v>
+      </c>
+      <c r="B115" t="s">
+        <v>5</v>
+      </c>
+      <c r="C115" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" s="1">
+        <v>111001801250</v>
+      </c>
+      <c r="B116" t="s">
+        <v>7</v>
+      </c>
+      <c r="C116" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" s="1">
+        <v>111001018325</v>
+      </c>
+      <c r="B117" t="s">
+        <v>7</v>
+      </c>
+      <c r="C117" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" s="1">
+        <v>111001800660</v>
+      </c>
+      <c r="B118" t="s">
+        <v>5</v>
+      </c>
+      <c r="C118" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" s="1">
+        <v>111001094439</v>
+      </c>
+      <c r="B119" t="s">
+        <v>7</v>
+      </c>
+      <c r="C119" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" s="1">
+        <v>111001034002</v>
+      </c>
+      <c r="B120" t="s">
+        <v>7</v>
+      </c>
+      <c r="C120" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" s="1">
+        <v>111001800457</v>
+      </c>
+      <c r="B121" t="s">
+        <v>5</v>
+      </c>
+      <c r="C121" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122" s="1">
+        <v>111001800163</v>
+      </c>
+      <c r="B122" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A123" s="1">
+        <v>111001106984</v>
+      </c>
+      <c r="B123" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A124" s="1">
+        <v>111001800384</v>
+      </c>
+      <c r="B124" t="s">
+        <v>5</v>
+      </c>
+      <c r="C124" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125" s="1">
+        <v>111001801098</v>
+      </c>
+      <c r="B125" t="s">
+        <v>7</v>
+      </c>
+      <c r="C125" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" s="1">
+        <v>111001107077</v>
+      </c>
+      <c r="B126" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" s="1">
+        <v>111001800392</v>
+      </c>
+      <c r="B127" t="s">
+        <v>5</v>
+      </c>
+      <c r="C127" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" s="1">
+        <v>111001801314</v>
+      </c>
+      <c r="B128" t="s">
+        <v>7</v>
+      </c>
+      <c r="C128" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129" s="1">
+        <v>111001107786</v>
+      </c>
+      <c r="B129" t="s">
+        <v>7</v>
+      </c>
+      <c r="C129" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{600A4391-AC9F-4D17-85AE-1F1D82F259AD}">
+  <dimension ref="B1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="47.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="6">
+        <v>503</v>
+      </c>
+      <c r="D1" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B2" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="8">
+        <v>301</v>
+      </c>
+      <c r="D2" s="6">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B3" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="6">
+        <v>301</v>
+      </c>
+      <c r="D3" s="6">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="6">
+        <v>301</v>
+      </c>
+      <c r="D4" s="6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="6">
+        <v>503</v>
+      </c>
+      <c r="D5" s="6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="8">
+        <v>501</v>
+      </c>
+      <c r="D6" s="6">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>